<commit_message>
remove the unneeded tab
</commit_message>
<xml_diff>
--- a/api/templates/export/contacts/en.xlsx
+++ b/api/templates/export/contacts/en.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25427"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\contacts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aepel\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DC6C14-D6E3-4357-B7AF-B000E88354DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>
-    <sheet name="Error Codes" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="144525"/>
   <extLst>
@@ -25,106 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="46">
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Run-time error</t>
-  </si>
-  <si>
-    <t>The actual temperature has drifted too far away from the setpoint</t>
-  </si>
-  <si>
-    <t>The temperature difference exceeds the limit</t>
-  </si>
-  <si>
-    <t>The internal instrument temperature was out of range</t>
-  </si>
-  <si>
-    <t>Optic signal of from detector exceeded the limit</t>
-  </si>
-  <si>
-    <t>Detector dark signal exceeded the limit</t>
-  </si>
-  <si>
-    <t>The power supply was detected to be out of range</t>
-  </si>
-  <si>
-    <t>The measured temperature of the optical system was not within the acceptable range</t>
-  </si>
-  <si>
-    <t>A valve positioning error was detected at the end of the run</t>
-  </si>
-  <si>
-    <t>Operation terminated error</t>
-  </si>
-  <si>
-    <t>Module is already running a test while performing command</t>
-  </si>
-  <si>
-    <t>Motion of the syringe drive was not detected</t>
-  </si>
-  <si>
-    <t>Syringe pressure reading exceeds the protocol limit</t>
-  </si>
-  <si>
-    <t>Syringe pressure reading is below the protocol limit</t>
-  </si>
-  <si>
-    <t>Cartridge loading error</t>
-  </si>
-  <si>
-    <t>Unable to initialize pressure sensor</t>
-  </si>
-  <si>
-    <t>The digital temperature reading for Thermistor A/Thermistor B/Ambient Thermistor/Optic Thermistor was not within the acceptable range</t>
-  </si>
-  <si>
-    <t>The system was unable to find the valve home position</t>
-  </si>
-  <si>
-    <t>Attempt to load a cartridge while the door is still closed</t>
-  </si>
-  <si>
-    <t>Failed to get to desired temperature</t>
-  </si>
-  <si>
-    <t>The system failed to find the plunger home position</t>
-  </si>
-  <si>
-    <t>The ultrasonic horn could not be tuned properly</t>
-  </si>
-  <si>
-    <t>The optical signal from Detector did not reach the expected value</t>
-  </si>
-  <si>
-    <t>The cartridge integrity test failed</t>
-  </si>
-  <si>
-    <t>Self-test error</t>
-  </si>
-  <si>
-    <t>Cooling fan operation was not verified. Measured temperature exceeded the limit</t>
-  </si>
-  <si>
-    <t>Post-run analysis error</t>
-  </si>
-  <si>
-    <t>Probe check failed. Probe check value was above the maximum</t>
-  </si>
-  <si>
-    <t>Probe check failed. Probe check value was below the minimum</t>
-  </si>
-  <si>
-    <t>Signal loss detected in the amplification curve</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>&lt;name&gt;</t>
   </si>
@@ -168,7 +69,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
@@ -349,18 +250,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -390,48 +287,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -459,7 +356,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -796,71 +693,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53.625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="33.25" style="3" customWidth="1"/>
-    <col min="3" max="3" width="26.125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="26" style="3" customWidth="1"/>
-    <col min="5" max="5" width="34.125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="53.58203125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="33.25" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.08203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26" style="2" customWidth="1"/>
+    <col min="5" max="5" width="34.08203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
-        <v>34</v>
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.5">
+      <c r="A1" s="8" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>45</v>
+    <row r="2" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="9" t="s">
-        <v>44</v>
+    <row r="3" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="7" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="5" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>35</v>
+    <row r="5" spans="1:5" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>42</v>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -871,316 +768,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
-        <v>1001</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>1002</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
-        <v>1004</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
-        <v>1005</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
-        <v>1006</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
-        <v>1007</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
-        <v>1017</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
-        <v>1018</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
-        <v>2003</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
-        <v>2005</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
-        <v>2008</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
-        <v>2009</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
-        <v>2011</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
-        <v>2014</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4">
-        <v>2016</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4">
-        <v>2018</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
-        <v>2022</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4">
-        <v>2025</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
-        <v>2032</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
-        <v>2034</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
-        <v>2037</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
-        <v>4010</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
-        <v>4017</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
-        <v>5006</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
-        <v>5007</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
-        <v>5011</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
[feat/HD-15591-Add-columns-in-contact-list] Fixed download report
</commit_message>
<xml_diff>
--- a/api/templates/export/contacts/en.xlsx
+++ b/api/templates/export/contacts/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25427"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10420"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aepel\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/export/contacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DC6C14-D6E3-4357-B7AF-B000E88354DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0061A49F-4DB2-3047-A231-883E35A5AF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="760" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>&lt;name&gt;</t>
   </si>
@@ -64,6 +64,24 @@
   </si>
   <si>
     <t>Printed date: &lt;date&gt;</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Cell</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>&lt;email&gt;</t>
+  </si>
+  <si>
+    <t>&lt;cell&gt;</t>
+  </si>
+  <si>
+    <t>&lt;phone&gt;</t>
   </si>
 </sst>
 </file>
@@ -136,7 +154,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -151,9 +169,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -166,9 +182,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -181,10 +195,10 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -196,10 +210,25 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -250,23 +279,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -276,59 +296,71 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -694,70 +726,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="53.58203125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="33.25" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.08203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="26" style="2" customWidth="1"/>
-    <col min="5" max="5" width="34.08203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="53.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="26" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" customWidth="1"/>
+    <col min="7" max="8" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" s="3" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="11" t="s">
         <v>5</v>
       </c>
+      <c r="F5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="F6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[feat/HD-15591-Add-columns-in-contact-list] Fixes, translated uk and fr templates.
</commit_message>
<xml_diff>
--- a/api/templates/export/contacts/en.xlsx
+++ b/api/templates/export/contacts/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/export/contacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0061A49F-4DB2-3047-A231-883E35A5AF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB888161-7E65-7745-8B9B-B1B10172C6FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="760" windowWidth="38620" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" r:id="rId1"/>
@@ -45,9 +45,6 @@
     <t>Tags</t>
   </si>
   <si>
-    <t>&lt;level&gt;</t>
-  </si>
-  <si>
     <t>&lt;state&gt;</t>
   </si>
   <si>
@@ -82,6 +79,9 @@
   </si>
   <si>
     <t>&lt;phone&gt;</t>
+  </si>
+  <si>
+    <t>&lt;assigments&gt;</t>
   </si>
 </sst>
 </file>
@@ -744,13 +744,13 @@
     </row>
     <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -764,19 +764,19 @@
         <v>4</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="12" t="s">
         <v>14</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -784,25 +784,25 @@
         <v>0</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>9</v>
-      </c>
       <c r="F6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>17</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
[feat/HD-15591-Add-columns-in-contact-list] Added Last Login column to List and Report
</commit_message>
<xml_diff>
--- a/api/templates/export/contacts/en.xlsx
+++ b/api/templates/export/contacts/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/export/contacts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB888161-7E65-7745-8B9B-B1B10172C6FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B3808F-C362-724D-9D0F-9013198EBF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21100" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>&lt;name&gt;</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>&lt;assigments&gt;</t>
+  </si>
+  <si>
+    <t>Last Login</t>
+  </si>
+  <si>
+    <t>&lt;lastLogin&gt;</t>
   </si>
 </sst>
 </file>
@@ -726,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.5" style="4" customWidth="1"/>
@@ -735,25 +741,26 @@
     <col min="5" max="5" width="34" style="1" customWidth="1"/>
     <col min="6" max="6" width="28.6640625" customWidth="1"/>
     <col min="7" max="8" width="18.33203125" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="4" spans="1:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" s="2" customFormat="1" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>2</v>
       </c>
@@ -775,11 +782,14 @@
       <c r="G5" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="11" t="s">
         <v>14</v>
       </c>
+      <c r="I5" s="12" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="6" spans="1:8" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
@@ -804,8 +814,11 @@
       <c r="H6" s="9" t="s">
         <v>17</v>
       </c>
+      <c r="I6" s="9" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>

</xml_diff>